<commit_message>
Se agrega la estimación de ángulo y velocidad angular. switches de fin de carrera y el momento dimensional del NACA 0012.
</commit_message>
<xml_diff>
--- a/04_CFD/00_XFLR5/Simpson/NACA_0012/tabla_hinge_moment_simpson_naca0012.xlsx
+++ b/04_CFD/00_XFLR5/Simpson/NACA_0012/tabla_hinge_moment_simpson_naca0012.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://udeconce-my.sharepoint.com/personal/joarriagada2021_udec_cl/Documents/Escritorio/Memoria/04_CFD/00_XFLR5/Simpson/NACA_0012/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_FDA9C290E5C67CE1C106BEE2347D6BBC2D477D51" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10849D88-7BBD-49DD-972A-E954B6D0544B}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="11_FDA9C290E5C67CE1C106BEE2347D6BBC2D477D51" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{897D6134-B355-40B0-B96E-CCC540F73312}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos (largo, corregido)" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,25 @@
     <sheet name="Verif Ch_alpha" sheetId="3" r:id="rId3"/>
     <sheet name="Verif Ch_delta" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
   <si>
     <t>archivo</t>
   </si>
@@ -176,6 +189,27 @@
   </si>
   <si>
     <t>Ch_a_alpha0</t>
+  </si>
+  <si>
+    <t>rho [kg/m^3]</t>
+  </si>
+  <si>
+    <t>V [m/s]</t>
+  </si>
+  <si>
+    <t>q [kg/ms^2]</t>
+  </si>
+  <si>
+    <t>c_ctrl [m]</t>
+  </si>
+  <si>
+    <t>S_ctrl [m^2]</t>
+  </si>
+  <si>
+    <t>K [Nm]</t>
+  </si>
+  <si>
+    <t>H [Nm]</t>
   </si>
 </sst>
 </file>
@@ -211,8 +245,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -515,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" bestFit="1" customWidth="1"/>
@@ -528,9 +563,15 @@
     <col min="9" max="9" width="7" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="12" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -564,8 +605,29 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M1" t="s">
+        <v>52</v>
+      </c>
+      <c r="N1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P1" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -599,8 +661,33 @@
       <c r="K2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M2" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N2">
+        <f>O2*1.602</f>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O2">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P2">
+        <f>0.5*L2*M2^2</f>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q2">
+        <f>P2*N2*O2</f>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R2">
+        <f>F2*Q2</f>
+        <v>11.201198401797981</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -634,8 +721,33 @@
       <c r="K3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L3" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M3" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N37" si="0">O3*1.602</f>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O3">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P3">
+        <f t="shared" ref="P3:P37" si="1">0.5*L3*M3^2</f>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" ref="Q3:Q37" si="2">P3*N3*O3</f>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R3">
+        <f t="shared" ref="R3:R37" si="3">F3*Q3</f>
+        <v>13.181645648645274</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -669,8 +781,33 @@
       <c r="K4" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M4" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O4">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R4">
+        <f t="shared" si="3"/>
+        <v>15.107286053190162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -704,8 +841,33 @@
       <c r="K5" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L5" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M5" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O5">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R5">
+        <f t="shared" si="3"/>
+        <v>16.968918466724933</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -739,8 +901,33 @@
       <c r="K6" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L6" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M6" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O6">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R6">
+        <f t="shared" si="3"/>
+        <v>18.757141715569983</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -774,8 +961,33 @@
       <c r="K7" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L7" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M7" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O7">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R7">
+        <f t="shared" si="3"/>
+        <v>20.463554750905235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -809,8 +1021,33 @@
       <c r="K8" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L8" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M8" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O8">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="3"/>
+        <v>22.079756523910607</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -844,8 +1081,33 @@
       <c r="K9" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L9" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M9" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O9">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="3"/>
+        <v>23.597746035709829</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -879,8 +1141,33 @@
       <c r="K10" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M10" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O10">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="3"/>
+        <v>25.010322387314279</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -914,8 +1201,33 @@
       <c r="K11" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L11" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M11" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O11">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="3"/>
+        <v>1.0221276064427518</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -949,8 +1261,33 @@
       <c r="K12" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L12" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M12" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O12">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="3"/>
+        <v>2.9897732550880263</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -984,8 +1321,33 @@
       <c r="K13" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L13" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M13" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O13">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="3"/>
+        <v>4.9468175802222509</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1019,8 +1381,33 @@
       <c r="K14" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L14" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M14" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O14">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="3"/>
+        <v>6.884059433137721</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1054,8 +1441,33 @@
       <c r="K15" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L15" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M15" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O15">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="3"/>
+        <v>8.792097640154827</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1089,8 +1501,33 @@
       <c r="K16" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L16" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M16" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O16">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="3"/>
+        <v>10.661130977650146</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1124,8 +1561,33 @@
       <c r="K17" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L17" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M17" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O17">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="3"/>
+        <v>12.48255837183169</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1159,8 +1621,33 @@
       <c r="K18" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L18" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M18" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O18">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="3"/>
+        <v>14.247178673991762</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1194,8 +1681,33 @@
       <c r="K19" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L19" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M19" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O19">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="3"/>
+        <v>15.946790860282187</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1229,8 +1741,33 @@
       <c r="K20" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L20" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M20" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N20">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O20">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="3"/>
+        <v>-3.6874603570982636</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -1264,8 +1801,33 @@
       <c r="K21" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L21" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M21" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O21">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="3"/>
+        <v>-1.7694209014858289</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -1299,8 +1861,33 @@
       <c r="K22" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L22" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M22" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N22">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O22">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R22">
+        <f t="shared" si="3"/>
+        <v>0.15901985266575105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>32</v>
       </c>
@@ -1334,8 +1921,33 @@
       <c r="K23" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L23" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M23" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N23">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O23">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P23">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q23">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R23">
+        <f t="shared" si="3"/>
+        <v>2.088460731676864</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -1369,8 +1981,33 @@
       <c r="K24" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L24" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M24" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N24">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O24">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P24">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q24">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R24">
+        <f t="shared" si="3"/>
+        <v>4.0095005618679007</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -1404,8 +2041,33 @@
       <c r="K25" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L25" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M25" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N25">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O25">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P25">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q25">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R25">
+        <f t="shared" si="3"/>
+        <v>5.9129381945311543</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -1439,8 +2101,33 @@
       <c r="K26" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L26" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M26" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N26">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O26">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P26">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q26">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R26">
+        <f t="shared" si="3"/>
+        <v>7.7895724809589213</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>36</v>
       </c>
@@ -1474,8 +2161,33 @@
       <c r="K27" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L27" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M27" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N27">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O27">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P27">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q27">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R27">
+        <f t="shared" si="3"/>
+        <v>9.6298022224996878</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1509,8 +2221,33 @@
       <c r="K28" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L28" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M28" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N28">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O28">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P28">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q28">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R28">
+        <f t="shared" si="3"/>
+        <v>11.425226370333379</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -1544,8 +2281,33 @@
       <c r="K29" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L29" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M29" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N29">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O29">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P29">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q29">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R29">
+        <f t="shared" si="3"/>
+        <v>-7.5573434885753557</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>39</v>
       </c>
@@ -1579,8 +2341,33 @@
       <c r="K30" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L30" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M30" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N30">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O30">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P30">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q30">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R30">
+        <f t="shared" si="3"/>
+        <v>-5.7023118991134973</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>40</v>
       </c>
@@ -1614,8 +2401,33 @@
       <c r="K31" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L31" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M31" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N31">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O31">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P31">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q31">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R31">
+        <f t="shared" si="3"/>
+        <v>-3.8194768385566236</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -1649,8 +2461,33 @@
       <c r="K32" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L32" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M32" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N32">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O32">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P32">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q32">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R32">
+        <f t="shared" si="3"/>
+        <v>-1.9180394556124363</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -1684,8 +2521,33 @@
       <c r="K33" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L33" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M33" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N33">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O33">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P33">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q33">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R33">
+        <f t="shared" si="3"/>
+        <v>-7.400923960544389E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -1719,8 +2581,33 @@
       <c r="K34" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L34" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M34" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N34">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O34">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P34">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q34">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R34">
+        <f t="shared" si="3"/>
+        <v>1.9034376326632543</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>44</v>
       </c>
@@ -1754,8 +2641,33 @@
       <c r="K35" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L35" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M35" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N35">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O35">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P35">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q35">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R35">
+        <f t="shared" si="3"/>
+        <v>3.8048750156074433</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>45</v>
       </c>
@@ -1789,8 +2701,33 @@
       <c r="K36" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L36" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M36" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N36">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O36">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P36">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q36">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R36">
+        <f t="shared" si="3"/>
+        <v>5.6877100761643167</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>46</v>
       </c>
@@ -1823,6 +2760,31 @@
       </c>
       <c r="K37" t="b">
         <v>1</v>
+      </c>
+      <c r="L37" s="1">
+        <v>1.522</v>
+      </c>
+      <c r="M37" s="1">
+        <v>170.15</v>
+      </c>
+      <c r="N37">
+        <f t="shared" si="0"/>
+        <v>0.15259050000000002</v>
+      </c>
+      <c r="O37">
+        <v>9.5250000000000001E-2</v>
+      </c>
+      <c r="P37">
+        <f t="shared" si="1"/>
+        <v>22031.728122500001</v>
+      </c>
+      <c r="Q37">
+        <f t="shared" si="2"/>
+        <v>320.21453705977109</v>
+      </c>
+      <c r="R37">
+        <f t="shared" si="3"/>
+        <v>7.5429416905980782</v>
       </c>
     </row>
   </sheetData>

</xml_diff>